<commit_message>
test(e2e): drop-to-sampling full flow + Phase 2 complete
E2E test verifies entire Phase 2 pipeline: project creation → ingest
(ledger+fs+rp+allowance) → AR/AP sampling design → state aggregation.

Fixture build_dummy.py: AR050-054 잔액 고정(충당금명세와 정합). 부실거래처가
랜덤화된 ledger 잔액 대비 부분충당으로 분류되어 표본에 포함되는 회귀를 차단.

- 135 tests pass (unit + integration + e2e)
- domain layer pure (no flask/sqlalchemy/pandas/openpyxl/pdfplumber)
</commit_message>
<xml_diff>
--- a/CC_SAMPLING_TOOL_V2/tests/e2e/fixtures/dummy_ledger.xlsx
+++ b/CC_SAMPLING_TOOL_V2/tests/e2e/fixtures/dummy_ledger.xlsx
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>516598</v>
+        <v>500000</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1894,7 +1894,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1351287</v>
+        <v>800000</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>8273</v>
+        <v>200000</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>69401</v>
+        <v>600000</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>54842</v>
+        <v>400000</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: party aggregation + AP activity-based PPS (ISA 505 완전성)
A) Account에 debit_amt·credit_amt 필드 추가 (당기 증가/감소)
B) ingest 시 party_id별 잔액·차변·대변 합산 (다중 시트 동일 거래처 1행 통합)
C) AP design은 잔액 대신 차변(당기증가) 기반 PPS — 활발히 거래했으나
   기말잔액 작은 거래처 누락 위험(부채 과소계상) 방지

- domain/sampling/{mus,stratified,allocation}.py: weight_attr 파라미터 추가
- application/ingest_uc.py: _aggregate_by_party helper, name·src_sheet 통합
- application/design_sampling_uc.py: kind==AP → weight_attr="debit_amt"
- configs/schema_mapping/default_aliases.yaml: 차변/대변 alias
- infrastructure/db/models.py·repository.py: debit_amt·credit_amt 컬럼·매핑
- tests/integration: test_party_aggregation, test_ap_activity_pps
- tests/e2e/fixtures/build_dummy.py: 차변/대변 컬럼 포함하도록 갱신

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CC_SAMPLING_TOOL_V2/tests/e2e/fixtures/dummy_ledger.xlsx
+++ b/CC_SAMPLING_TOOL_V2/tests/e2e/fixtures/dummy_ledger.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,16 @@
           <t>환율</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -476,6 +486,12 @@
       <c r="F2" t="n">
         <v>1300</v>
       </c>
+      <c r="G2" t="n">
+        <v>687868</v>
+      </c>
+      <c r="H2" t="n">
+        <v>320749</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -494,7 +510,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>738201</v>
+        <v>1282390</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -504,6 +520,12 @@
       <c r="F3" t="n">
         <v>1300</v>
       </c>
+      <c r="G3" t="n">
+        <v>5554227</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6006669</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -522,7 +544,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>17319</v>
+        <v>27812</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -532,6 +554,12 @@
       <c r="F4" t="n">
         <v>1300</v>
       </c>
+      <c r="G4" t="n">
+        <v>103867</v>
+      </c>
+      <c r="H4" t="n">
+        <v>48518</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -550,7 +578,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10485</v>
+        <v>13266</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -560,6 +588,12 @@
       <c r="F5" t="n">
         <v>1300</v>
       </c>
+      <c r="G5" t="n">
+        <v>29668</v>
+      </c>
+      <c r="H5" t="n">
+        <v>46153</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -578,7 +612,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18646</v>
+        <v>72297</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -588,6 +622,12 @@
       <c r="F6" t="n">
         <v>1300</v>
       </c>
+      <c r="G6" t="n">
+        <v>313189</v>
+      </c>
+      <c r="H6" t="n">
+        <v>124099</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -606,7 +646,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>27812</v>
+        <v>2190041</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -615,6 +655,12 @@
       </c>
       <c r="F7" t="n">
         <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>12932239</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3642125</v>
       </c>
     </row>
     <row r="8">
@@ -634,7 +680,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>563629</v>
+        <v>46721</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -643,6 +689,12 @@
       </c>
       <c r="F8" t="n">
         <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>120400</v>
+      </c>
+      <c r="H8" t="n">
+        <v>89343</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +714,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31803</v>
+        <v>134039</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -671,6 +723,12 @@
       </c>
       <c r="F9" t="n">
         <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>633736</v>
+      </c>
+      <c r="H9" t="n">
+        <v>249405</v>
       </c>
     </row>
     <row r="10">
@@ -690,7 +748,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>294333</v>
+        <v>2916740</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -699,6 +757,12 @@
       </c>
       <c r="F10" t="n">
         <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10178229</v>
+      </c>
+      <c r="H10" t="n">
+        <v>9966810</v>
       </c>
     </row>
     <row r="11">
@@ -718,7 +782,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1371406</v>
+        <v>13466</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -727,6 +791,12 @@
       </c>
       <c r="F11" t="n">
         <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>60272</v>
+      </c>
+      <c r="H11" t="n">
+        <v>43594</v>
       </c>
     </row>
     <row r="12">
@@ -746,7 +816,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>72297</v>
+        <v>2282777</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -755,6 +825,12 @@
       </c>
       <c r="F12" t="n">
         <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>7434065</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8102640</v>
       </c>
     </row>
     <row r="13">
@@ -774,7 +850,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3843127</v>
+        <v>521187</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -783,6 +859,12 @@
       </c>
       <c r="F13" t="n">
         <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1560280</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1109702</v>
       </c>
     </row>
     <row r="14">
@@ -802,7 +884,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2756624</v>
+        <v>31139</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -811,6 +893,12 @@
       </c>
       <c r="F14" t="n">
         <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>99676</v>
+      </c>
+      <c r="H14" t="n">
+        <v>100670</v>
       </c>
     </row>
     <row r="15">
@@ -830,7 +918,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>19644</v>
+        <v>159417</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -839,6 +927,12 @@
       </c>
       <c r="F15" t="n">
         <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>502442</v>
+      </c>
+      <c r="H15" t="n">
+        <v>786022</v>
       </c>
     </row>
     <row r="16">
@@ -858,7 +952,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>13350</v>
+        <v>12679</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -867,6 +961,12 @@
       </c>
       <c r="F16" t="n">
         <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>33724</v>
+      </c>
+      <c r="H16" t="n">
+        <v>34198</v>
       </c>
     </row>
     <row r="17">
@@ -886,7 +986,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>46721</v>
+        <v>566274</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -895,6 +995,12 @@
       </c>
       <c r="F17" t="n">
         <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3311612</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1003251</v>
       </c>
     </row>
     <row r="18">
@@ -914,7 +1020,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>65551</v>
+        <v>2719078</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -923,6 +1029,12 @@
       </c>
       <c r="F18" t="n">
         <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>14960125</v>
+      </c>
+      <c r="H18" t="n">
+        <v>7064480</v>
       </c>
     </row>
     <row r="19">
@@ -942,7 +1054,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1925445</v>
+        <v>10252676</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -951,6 +1063,12 @@
       </c>
       <c r="F19" t="n">
         <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>40874334</v>
+      </c>
+      <c r="H19" t="n">
+        <v>43974977</v>
       </c>
     </row>
     <row r="20">
@@ -970,7 +1088,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>7710896</v>
+        <v>17600</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -979,6 +1097,12 @@
       </c>
       <c r="F20" t="n">
         <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>101703</v>
+      </c>
+      <c r="H20" t="n">
+        <v>55603</v>
       </c>
     </row>
     <row r="21">
@@ -998,7 +1122,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2713613</v>
+        <v>5975000</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1007,6 +1131,12 @@
       </c>
       <c r="F21" t="n">
         <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>29424706</v>
+      </c>
+      <c r="H21" t="n">
+        <v>15437163</v>
       </c>
     </row>
     <row r="22">
@@ -1026,7 +1156,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>52930</v>
+        <v>3979288</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1035,6 +1165,12 @@
       </c>
       <c r="F22" t="n">
         <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>21041277</v>
+      </c>
+      <c r="H22" t="n">
+        <v>9932638</v>
       </c>
     </row>
     <row r="23">
@@ -1054,7 +1190,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3136332</v>
+        <v>915280</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1063,6 +1199,12 @@
       </c>
       <c r="F23" t="n">
         <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>3100989</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4386270</v>
       </c>
     </row>
     <row r="24">
@@ -1082,7 +1224,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1178804</v>
+        <v>75207</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1091,6 +1233,12 @@
       </c>
       <c r="F24" t="n">
         <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>185640</v>
+      </c>
+      <c r="H24" t="n">
+        <v>128329</v>
       </c>
     </row>
     <row r="25">
@@ -1110,7 +1258,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>62231</v>
+        <v>69401</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1119,6 +1267,12 @@
       </c>
       <c r="F25" t="n">
         <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>207541</v>
+      </c>
+      <c r="H25" t="n">
+        <v>199065</v>
       </c>
     </row>
     <row r="26">
@@ -1138,7 +1292,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2282777</v>
+        <v>310436</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1147,6 +1301,12 @@
       </c>
       <c r="F26" t="n">
         <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1178648</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1062635</v>
       </c>
     </row>
     <row r="27">
@@ -1166,7 +1326,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>119840</v>
+        <v>86446</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1175,6 +1335,12 @@
       </c>
       <c r="F27" t="n">
         <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>471644</v>
+      </c>
+      <c r="H27" t="n">
+        <v>213908</v>
       </c>
     </row>
     <row r="28">
@@ -1194,7 +1360,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>521187</v>
+        <v>989850</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1203,6 +1369,12 @@
       </c>
       <c r="F28" t="n">
         <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4682875</v>
+      </c>
+      <c r="H28" t="n">
+        <v>2802805</v>
       </c>
     </row>
     <row r="29">
@@ -1222,7 +1394,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>84578</v>
+        <v>36319</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1231,6 +1403,12 @@
       </c>
       <c r="F29" t="n">
         <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>98238</v>
+      </c>
+      <c r="H29" t="n">
+        <v>83964</v>
       </c>
     </row>
     <row r="30">
@@ -1250,7 +1428,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>16697444</v>
+        <v>25905</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1259,6 +1437,12 @@
       </c>
       <c r="F30" t="n">
         <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>137926</v>
+      </c>
+      <c r="H30" t="n">
+        <v>55389</v>
       </c>
     </row>
     <row r="31">
@@ -1278,7 +1462,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>13616</v>
+        <v>50614</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1287,6 +1471,12 @@
       </c>
       <c r="F31" t="n">
         <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>186046</v>
+      </c>
+      <c r="H31" t="n">
+        <v>141334</v>
       </c>
     </row>
     <row r="32">
@@ -1306,7 +1496,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2485349</v>
+        <v>1955835</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1315,6 +1505,12 @@
       </c>
       <c r="F32" t="n">
         <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4893433</v>
+      </c>
+      <c r="H32" t="n">
+        <v>8815353</v>
       </c>
     </row>
     <row r="33">
@@ -1334,7 +1530,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>159417</v>
+        <v>2964899</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1343,6 +1539,12 @@
       </c>
       <c r="F33" t="n">
         <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>14703348</v>
+      </c>
+      <c r="H33" t="n">
+        <v>9186009</v>
       </c>
     </row>
     <row r="34">
@@ -1362,7 +1564,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>141344</v>
+        <v>16968097</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1371,6 +1573,12 @@
       </c>
       <c r="F34" t="n">
         <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>60567887</v>
+      </c>
+      <c r="H34" t="n">
+        <v>49146835</v>
       </c>
     </row>
     <row r="35">
@@ -1390,7 +1598,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6771</v>
+        <v>12223</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1399,6 +1607,12 @@
       </c>
       <c r="F35" t="n">
         <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>44024</v>
+      </c>
+      <c r="H35" t="n">
+        <v>26489</v>
       </c>
     </row>
     <row r="36">
@@ -1418,7 +1632,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>373722</v>
+        <v>58047</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1427,6 +1641,12 @@
       </c>
       <c r="F36" t="n">
         <v>1</v>
+      </c>
+      <c r="G36" t="n">
+        <v>141618</v>
+      </c>
+      <c r="H36" t="n">
+        <v>209117</v>
       </c>
     </row>
     <row r="37">
@@ -1446,7 +1666,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>72798</v>
+        <v>5003</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1455,6 +1675,12 @@
       </c>
       <c r="F37" t="n">
         <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>13034</v>
+      </c>
+      <c r="H37" t="n">
+        <v>9282</v>
       </c>
     </row>
     <row r="38">
@@ -1474,7 +1700,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>566274</v>
+        <v>142061</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1483,6 +1709,12 @@
       </c>
       <c r="F38" t="n">
         <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>324077</v>
+      </c>
+      <c r="H38" t="n">
+        <v>316487</v>
       </c>
     </row>
     <row r="39">
@@ -1502,7 +1734,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6164307</v>
+        <v>361413</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1511,6 +1743,12 @@
       </c>
       <c r="F39" t="n">
         <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1087503</v>
+      </c>
+      <c r="H39" t="n">
+        <v>981548</v>
       </c>
     </row>
     <row r="40">
@@ -1530,7 +1768,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2719078</v>
+        <v>121123</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1539,6 +1777,12 @@
       </c>
       <c r="F40" t="n">
         <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>298133</v>
+      </c>
+      <c r="H40" t="n">
+        <v>388591</v>
       </c>
     </row>
     <row r="41">
@@ -1558,7 +1802,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>101018</v>
+        <v>610296</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1567,6 +1811,12 @@
       </c>
       <c r="F41" t="n">
         <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1981882</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1223285</v>
       </c>
     </row>
     <row r="42">
@@ -1586,7 +1836,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>139155</v>
+        <v>10139538</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1595,6 +1845,12 @@
       </c>
       <c r="F42" t="n">
         <v>1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>31017125</v>
+      </c>
+      <c r="H42" t="n">
+        <v>44624042</v>
       </c>
     </row>
     <row r="43">
@@ -1614,7 +1870,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3390676</v>
+        <v>63725</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1623,6 +1879,12 @@
       </c>
       <c r="F43" t="n">
         <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>179760</v>
+      </c>
+      <c r="H43" t="n">
+        <v>307924</v>
       </c>
     </row>
     <row r="44">
@@ -1642,7 +1904,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>17600</v>
+        <v>71990</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1651,6 +1913,12 @@
       </c>
       <c r="F44" t="n">
         <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>300394</v>
+      </c>
+      <c r="H44" t="n">
+        <v>114799</v>
       </c>
     </row>
     <row r="45">
@@ -1670,7 +1938,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>121115</v>
+        <v>1894269</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1679,6 +1947,12 @@
       </c>
       <c r="F45" t="n">
         <v>1</v>
+      </c>
+      <c r="G45" t="n">
+        <v>8659970</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3444798</v>
       </c>
     </row>
     <row r="46">
@@ -1698,7 +1972,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5975000</v>
+        <v>127760</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1707,6 +1981,12 @@
       </c>
       <c r="F46" t="n">
         <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>719674</v>
+      </c>
+      <c r="H46" t="n">
+        <v>350692</v>
       </c>
     </row>
     <row r="47">
@@ -1726,7 +2006,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15522380</v>
+        <v>64944</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1735,6 +2015,12 @@
       </c>
       <c r="F47" t="n">
         <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>332270</v>
+      </c>
+      <c r="H47" t="n">
+        <v>172351</v>
       </c>
     </row>
     <row r="48">
@@ -1754,7 +2040,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>13669193</v>
+        <v>70992</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1763,6 +2049,12 @@
       </c>
       <c r="F48" t="n">
         <v>1</v>
+      </c>
+      <c r="G48" t="n">
+        <v>365865</v>
+      </c>
+      <c r="H48" t="n">
+        <v>294910</v>
       </c>
     </row>
     <row r="49">
@@ -1782,7 +2074,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>17328872</v>
+        <v>85456</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1791,6 +2083,12 @@
       </c>
       <c r="F49" t="n">
         <v>1</v>
+      </c>
+      <c r="G49" t="n">
+        <v>450637</v>
+      </c>
+      <c r="H49" t="n">
+        <v>349477</v>
       </c>
     </row>
     <row r="50">
@@ -1810,7 +2108,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>157494</v>
+        <v>39994</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1819,6 +2117,12 @@
       </c>
       <c r="F50" t="n">
         <v>1</v>
+      </c>
+      <c r="G50" t="n">
+        <v>158821</v>
+      </c>
+      <c r="H50" t="n">
+        <v>162316</v>
       </c>
     </row>
     <row r="51">
@@ -1838,7 +2142,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>10205079</v>
+        <v>16852</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1847,6 +2151,12 @@
       </c>
       <c r="F51" t="n">
         <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>65536</v>
+      </c>
+      <c r="H51" t="n">
+        <v>36699</v>
       </c>
     </row>
     <row r="52">
@@ -1876,6 +2186,12 @@
       <c r="F52" t="n">
         <v>1</v>
       </c>
+      <c r="G52" t="n">
+        <v>1894455</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2389787</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1904,6 +2220,12 @@
       <c r="F53" t="n">
         <v>1</v>
       </c>
+      <c r="G53" t="n">
+        <v>2766835</v>
+      </c>
+      <c r="H53" t="n">
+        <v>1817295</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1932,6 +2254,12 @@
       <c r="F54" t="n">
         <v>1</v>
       </c>
+      <c r="G54" t="n">
+        <v>670190</v>
+      </c>
+      <c r="H54" t="n">
+        <v>637857</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1960,6 +2288,12 @@
       <c r="F55" t="n">
         <v>1</v>
       </c>
+      <c r="G55" t="n">
+        <v>2350736</v>
+      </c>
+      <c r="H55" t="n">
+        <v>2271254</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1988,6 +2322,12 @@
       <c r="F56" t="n">
         <v>1</v>
       </c>
+      <c r="G56" t="n">
+        <v>1856937</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1873688</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2006,7 +2346,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>310436</v>
+        <v>16252107</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2015,6 +2355,12 @@
       </c>
       <c r="F57" t="n">
         <v>1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>63580371</v>
+      </c>
+      <c r="H57" t="n">
+        <v>34532900</v>
       </c>
     </row>
     <row r="58">
@@ -2034,7 +2380,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>551233</v>
+        <v>9987758</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2043,6 +2389,12 @@
       </c>
       <c r="F58" t="n">
         <v>1</v>
+      </c>
+      <c r="G58" t="n">
+        <v>51969244</v>
+      </c>
+      <c r="H58" t="n">
+        <v>48948010</v>
       </c>
     </row>
     <row r="59">
@@ -2062,7 +2414,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>182508</v>
+        <v>597370</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2071,6 +2423,12 @@
       </c>
       <c r="F59" t="n">
         <v>1</v>
+      </c>
+      <c r="G59" t="n">
+        <v>2970968</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1073604</v>
       </c>
     </row>
     <row r="60">
@@ -2090,7 +2448,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>897988</v>
+        <v>37750</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2099,6 +2457,12 @@
       </c>
       <c r="F60" t="n">
         <v>1</v>
+      </c>
+      <c r="G60" t="n">
+        <v>94683</v>
+      </c>
+      <c r="H60" t="n">
+        <v>76596</v>
       </c>
     </row>
     <row r="61">
@@ -2118,7 +2482,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>155960</v>
+        <v>854876</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2127,6 +2491,12 @@
       </c>
       <c r="F61" t="n">
         <v>1</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2209597</v>
+      </c>
+      <c r="H61" t="n">
+        <v>3755290</v>
       </c>
     </row>
     <row r="62">
@@ -2146,7 +2516,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>152408</v>
+        <v>742951</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2155,6 +2525,12 @@
       </c>
       <c r="F62" t="n">
         <v>1</v>
+      </c>
+      <c r="G62" t="n">
+        <v>2527245</v>
+      </c>
+      <c r="H62" t="n">
+        <v>2541124</v>
       </c>
     </row>
     <row r="63">
@@ -2174,7 +2550,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>968298</v>
+        <v>26605</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2183,6 +2559,12 @@
       </c>
       <c r="F63" t="n">
         <v>1</v>
+      </c>
+      <c r="G63" t="n">
+        <v>138276</v>
+      </c>
+      <c r="H63" t="n">
+        <v>107544</v>
       </c>
     </row>
     <row r="64">
@@ -2202,7 +2584,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>31224</v>
+        <v>12899</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2211,6 +2593,12 @@
       </c>
       <c r="F64" t="n">
         <v>1</v>
+      </c>
+      <c r="G64" t="n">
+        <v>73968</v>
+      </c>
+      <c r="H64" t="n">
+        <v>38933</v>
       </c>
     </row>
     <row r="65">
@@ -2230,7 +2618,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>42397</v>
+        <v>86962</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2239,6 +2627,12 @@
       </c>
       <c r="F65" t="n">
         <v>1</v>
+      </c>
+      <c r="G65" t="n">
+        <v>247334</v>
+      </c>
+      <c r="H65" t="n">
+        <v>207092</v>
       </c>
     </row>
     <row r="66">
@@ -2258,7 +2652,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>25905</v>
+        <v>125174</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2267,6 +2661,12 @@
       </c>
       <c r="F66" t="n">
         <v>1</v>
+      </c>
+      <c r="G66" t="n">
+        <v>632721</v>
+      </c>
+      <c r="H66" t="n">
+        <v>330581</v>
       </c>
     </row>
     <row r="67">
@@ -2286,7 +2686,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1547029</v>
+        <v>2257038</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2295,6 +2695,12 @@
       </c>
       <c r="F67" t="n">
         <v>1</v>
+      </c>
+      <c r="G67" t="n">
+        <v>5697428</v>
+      </c>
+      <c r="H67" t="n">
+        <v>10574356</v>
       </c>
     </row>
     <row r="68">
@@ -2314,7 +2720,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>50614</v>
+        <v>184656</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2323,6 +2729,12 @@
       </c>
       <c r="F68" t="n">
         <v>1</v>
+      </c>
+      <c r="G68" t="n">
+        <v>858630</v>
+      </c>
+      <c r="H68" t="n">
+        <v>803744</v>
       </c>
     </row>
     <row r="69">
@@ -2342,7 +2754,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>650943</v>
+        <v>2261885</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2351,6 +2763,12 @@
       </c>
       <c r="F69" t="n">
         <v>1</v>
+      </c>
+      <c r="G69" t="n">
+        <v>12826887</v>
+      </c>
+      <c r="H69" t="n">
+        <v>7364180</v>
       </c>
     </row>
     <row r="70">
@@ -2370,7 +2788,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>2699024</v>
+        <v>1455509</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2379,6 +2797,12 @@
       </c>
       <c r="F70" t="n">
         <v>1</v>
+      </c>
+      <c r="G70" t="n">
+        <v>5883442</v>
+      </c>
+      <c r="H70" t="n">
+        <v>6629582</v>
       </c>
     </row>
     <row r="71">
@@ -2398,7 +2822,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>76787</v>
+        <v>70642</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2407,6 +2831,12 @@
       </c>
       <c r="F71" t="n">
         <v>1</v>
+      </c>
+      <c r="G71" t="n">
+        <v>360566</v>
+      </c>
+      <c r="H71" t="n">
+        <v>143000</v>
       </c>
     </row>
     <row r="72">
@@ -2426,7 +2856,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>3850672</v>
+        <v>60512</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2435,6 +2865,12 @@
       </c>
       <c r="F72" t="n">
         <v>1</v>
+      </c>
+      <c r="G72" t="n">
+        <v>296555</v>
+      </c>
+      <c r="H72" t="n">
+        <v>208625</v>
       </c>
     </row>
     <row r="73">
@@ -2454,7 +2890,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>15143001</v>
+        <v>152350</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2463,6 +2899,12 @@
       </c>
       <c r="F73" t="n">
         <v>1</v>
+      </c>
+      <c r="G73" t="n">
+        <v>628123</v>
+      </c>
+      <c r="H73" t="n">
+        <v>485798</v>
       </c>
     </row>
     <row r="74">
@@ -2482,7 +2924,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>11850</v>
+        <v>18248</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2491,6 +2933,12 @@
       </c>
       <c r="F74" t="n">
         <v>1</v>
+      </c>
+      <c r="G74" t="n">
+        <v>40645</v>
+      </c>
+      <c r="H74" t="n">
+        <v>39591</v>
       </c>
     </row>
     <row r="75">
@@ -2510,7 +2958,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>16968097</v>
+        <v>16584</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2519,6 +2967,12 @@
       </c>
       <c r="F75" t="n">
         <v>1</v>
+      </c>
+      <c r="G75" t="n">
+        <v>66847</v>
+      </c>
+      <c r="H75" t="n">
+        <v>57481</v>
       </c>
     </row>
     <row r="76">
@@ -2538,7 +2992,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>548552</v>
+        <v>11649</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2547,6 +3001,12 @@
       </c>
       <c r="F76" t="n">
         <v>1</v>
+      </c>
+      <c r="G76" t="n">
+        <v>51838</v>
+      </c>
+      <c r="H76" t="n">
+        <v>38085</v>
       </c>
     </row>
     <row r="77">
@@ -2566,7 +3026,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>327653</v>
+        <v>1598210</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2575,6 +3035,12 @@
       </c>
       <c r="F77" t="n">
         <v>1</v>
+      </c>
+      <c r="G77" t="n">
+        <v>4968422</v>
+      </c>
+      <c r="H77" t="n">
+        <v>5239805</v>
       </c>
     </row>
     <row r="78">
@@ -2594,7 +3060,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>11006639</v>
+        <v>630814</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2603,6 +3069,12 @@
       </c>
       <c r="F78" t="n">
         <v>1</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1886527</v>
+      </c>
+      <c r="H78" t="n">
+        <v>2101389</v>
       </c>
     </row>
     <row r="79">
@@ -2622,7 +3094,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>30051</v>
+        <v>188418</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2631,6 +3103,12 @@
       </c>
       <c r="F79" t="n">
         <v>1</v>
+      </c>
+      <c r="G79" t="n">
+        <v>1049678</v>
+      </c>
+      <c r="H79" t="n">
+        <v>416226</v>
       </c>
     </row>
     <row r="80">
@@ -2650,7 +3128,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>58047</v>
+        <v>352851</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2659,6 +3137,12 @@
       </c>
       <c r="F80" t="n">
         <v>1</v>
+      </c>
+      <c r="G80" t="n">
+        <v>877359</v>
+      </c>
+      <c r="H80" t="n">
+        <v>1075282</v>
       </c>
     </row>
     <row r="81">
@@ -2678,7 +3162,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>10101</v>
+        <v>15067</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2687,6 +3171,12 @@
       </c>
       <c r="F81" t="n">
         <v>1</v>
+      </c>
+      <c r="G81" t="n">
+        <v>55950</v>
+      </c>
+      <c r="H81" t="n">
+        <v>33817</v>
       </c>
     </row>
     <row r="82">
@@ -2706,7 +3196,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>6536</v>
+        <v>167590</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2715,6 +3205,12 @@
       </c>
       <c r="F82" t="n">
         <v>1</v>
+      </c>
+      <c r="G82" t="n">
+        <v>936513</v>
+      </c>
+      <c r="H82" t="n">
+        <v>341979</v>
       </c>
     </row>
     <row r="83">
@@ -2734,7 +3230,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1453795</v>
+        <v>14651870</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2743,6 +3239,12 @@
       </c>
       <c r="F83" t="n">
         <v>1</v>
+      </c>
+      <c r="G83" t="n">
+        <v>50764820</v>
+      </c>
+      <c r="H83" t="n">
+        <v>34957566</v>
       </c>
     </row>
     <row r="84">
@@ -2762,7 +3264,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>19234</v>
+        <v>97566</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2771,6 +3273,12 @@
       </c>
       <c r="F84" t="n">
         <v>1</v>
+      </c>
+      <c r="G84" t="n">
+        <v>280829</v>
+      </c>
+      <c r="H84" t="n">
+        <v>471610</v>
       </c>
     </row>
     <row r="85">
@@ -2790,7 +3298,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1076503</v>
+        <v>913700</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2799,6 +3307,12 @@
       </c>
       <c r="F85" t="n">
         <v>1</v>
+      </c>
+      <c r="G85" t="n">
+        <v>2422383</v>
+      </c>
+      <c r="H85" t="n">
+        <v>3506245</v>
       </c>
     </row>
     <row r="86">
@@ -2818,7 +3332,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>71055</v>
+        <v>37110</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2827,6 +3341,12 @@
       </c>
       <c r="F86" t="n">
         <v>1</v>
+      </c>
+      <c r="G86" t="n">
+        <v>138275</v>
+      </c>
+      <c r="H86" t="n">
+        <v>122634</v>
       </c>
     </row>
     <row r="87">
@@ -2846,7 +3366,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>72581</v>
+        <v>113191</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2855,6 +3375,12 @@
       </c>
       <c r="F87" t="n">
         <v>1</v>
+      </c>
+      <c r="G87" t="n">
+        <v>387846</v>
+      </c>
+      <c r="H87" t="n">
+        <v>206312</v>
       </c>
     </row>
     <row r="88">
@@ -2874,7 +3400,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>140342</v>
+        <v>52922</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2883,6 +3409,12 @@
       </c>
       <c r="F88" t="n">
         <v>1</v>
+      </c>
+      <c r="G88" t="n">
+        <v>223132</v>
+      </c>
+      <c r="H88" t="n">
+        <v>160969</v>
       </c>
     </row>
     <row r="89">
@@ -2902,7 +3434,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>342132</v>
+        <v>10765</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2911,6 +3443,12 @@
       </c>
       <c r="F89" t="n">
         <v>1</v>
+      </c>
+      <c r="G89" t="n">
+        <v>43811</v>
+      </c>
+      <c r="H89" t="n">
+        <v>27280</v>
       </c>
     </row>
     <row r="90">
@@ -2930,7 +3468,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>994827</v>
+        <v>6693</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2939,6 +3477,12 @@
       </c>
       <c r="F90" t="n">
         <v>1</v>
+      </c>
+      <c r="G90" t="n">
+        <v>37976</v>
+      </c>
+      <c r="H90" t="n">
+        <v>15393</v>
       </c>
     </row>
     <row r="91">
@@ -2958,7 +3502,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>610296</v>
+        <v>6261</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2967,6 +3511,12 @@
       </c>
       <c r="F91" t="n">
         <v>1</v>
+      </c>
+      <c r="G91" t="n">
+        <v>19332</v>
+      </c>
+      <c r="H91" t="n">
+        <v>29243</v>
       </c>
     </row>
     <row r="92">
@@ -2986,7 +3536,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>62883</v>
+        <v>45283</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2995,6 +3545,12 @@
       </c>
       <c r="F92" t="n">
         <v>1</v>
+      </c>
+      <c r="G92" t="n">
+        <v>114034</v>
+      </c>
+      <c r="H92" t="n">
+        <v>134849</v>
       </c>
     </row>
     <row r="93">
@@ -3014,7 +3570,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>16245</v>
+        <v>17284685</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -3023,6 +3579,12 @@
       </c>
       <c r="F93" t="n">
         <v>1</v>
+      </c>
+      <c r="G93" t="n">
+        <v>52449271</v>
+      </c>
+      <c r="H93" t="n">
+        <v>34963250</v>
       </c>
     </row>
     <row r="94">
@@ -3042,7 +3604,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>8971353</v>
+        <v>2711785</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -3051,6 +3613,12 @@
       </c>
       <c r="F94" t="n">
         <v>1</v>
+      </c>
+      <c r="G94" t="n">
+        <v>13021095</v>
+      </c>
+      <c r="H94" t="n">
+        <v>4916785</v>
       </c>
     </row>
     <row r="95">
@@ -3070,7 +3638,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>7421579</v>
+        <v>16994</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3079,6 +3647,12 @@
       </c>
       <c r="F95" t="n">
         <v>1</v>
+      </c>
+      <c r="G95" t="n">
+        <v>46450</v>
+      </c>
+      <c r="H95" t="n">
+        <v>78741</v>
       </c>
     </row>
     <row r="96">
@@ -3098,7 +3672,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>8078</v>
+        <v>190752</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3107,6 +3681,12 @@
       </c>
       <c r="F96" t="n">
         <v>1</v>
+      </c>
+      <c r="G96" t="n">
+        <v>865588</v>
+      </c>
+      <c r="H96" t="n">
+        <v>821323</v>
       </c>
     </row>
     <row r="97">
@@ -3126,7 +3706,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2085257</v>
+        <v>14123</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3135,6 +3715,12 @@
       </c>
       <c r="F97" t="n">
         <v>1</v>
+      </c>
+      <c r="G97" t="n">
+        <v>40809</v>
+      </c>
+      <c r="H97" t="n">
+        <v>34256</v>
       </c>
     </row>
     <row r="98">
@@ -3154,7 +3740,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>13147586</v>
+        <v>11807</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -3163,6 +3749,12 @@
       </c>
       <c r="F98" t="n">
         <v>1</v>
+      </c>
+      <c r="G98" t="n">
+        <v>39630</v>
+      </c>
+      <c r="H98" t="n">
+        <v>40564</v>
       </c>
     </row>
     <row r="99">
@@ -3182,7 +3774,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>16372</v>
+        <v>143256</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3191,6 +3783,12 @@
       </c>
       <c r="F99" t="n">
         <v>1</v>
+      </c>
+      <c r="G99" t="n">
+        <v>311269</v>
+      </c>
+      <c r="H99" t="n">
+        <v>570641</v>
       </c>
     </row>
     <row r="100">
@@ -3210,7 +3808,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>196775</v>
+        <v>19538</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -3219,6 +3817,12 @@
       </c>
       <c r="F100" t="n">
         <v>1</v>
+      </c>
+      <c r="G100" t="n">
+        <v>59544</v>
+      </c>
+      <c r="H100" t="n">
+        <v>41695</v>
       </c>
     </row>
     <row r="101">
@@ -3238,7 +3842,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>15443</v>
+        <v>144301</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -3247,6 +3851,12 @@
       </c>
       <c r="F101" t="n">
         <v>1</v>
+      </c>
+      <c r="G101" t="n">
+        <v>595145</v>
+      </c>
+      <c r="H101" t="n">
+        <v>320427</v>
       </c>
     </row>
     <row r="102">
@@ -3266,7 +3876,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>127760</v>
+        <v>625066</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3275,6 +3885,12 @@
       </c>
       <c r="F102" t="n">
         <v>1</v>
+      </c>
+      <c r="G102" t="n">
+        <v>1694930</v>
+      </c>
+      <c r="H102" t="n">
+        <v>1696745</v>
       </c>
     </row>
     <row r="103">
@@ -3294,7 +3910,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>51677</v>
+        <v>19917</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3303,6 +3919,12 @@
       </c>
       <c r="F103" t="n">
         <v>1</v>
+      </c>
+      <c r="G103" t="n">
+        <v>42779</v>
+      </c>
+      <c r="H103" t="n">
+        <v>31161</v>
       </c>
     </row>
     <row r="104">
@@ -3322,7 +3944,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>64944</v>
+        <v>2653147</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -3331,6 +3953,12 @@
       </c>
       <c r="F104" t="n">
         <v>1</v>
+      </c>
+      <c r="G104" t="n">
+        <v>7316919</v>
+      </c>
+      <c r="H104" t="n">
+        <v>8388356</v>
       </c>
     </row>
     <row r="105">
@@ -3350,7 +3978,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1988995</v>
+        <v>329711</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3359,6 +3987,12 @@
       </c>
       <c r="F105" t="n">
         <v>1</v>
+      </c>
+      <c r="G105" t="n">
+        <v>1739450</v>
+      </c>
+      <c r="H105" t="n">
+        <v>993294</v>
       </c>
     </row>
     <row r="106">
@@ -3378,7 +4012,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>70992</v>
+        <v>659430</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3387,6 +4021,12 @@
       </c>
       <c r="F106" t="n">
         <v>1</v>
+      </c>
+      <c r="G106" t="n">
+        <v>3663069</v>
+      </c>
+      <c r="H106" t="n">
+        <v>3228629</v>
       </c>
     </row>
     <row r="107">
@@ -3406,7 +4046,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>85456</v>
+        <v>153161</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3415,6 +4055,12 @@
       </c>
       <c r="F107" t="n">
         <v>1</v>
+      </c>
+      <c r="G107" t="n">
+        <v>908210</v>
+      </c>
+      <c r="H107" t="n">
+        <v>413454</v>
       </c>
     </row>
     <row r="108">
@@ -3434,7 +4080,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>804905</v>
+        <v>15932663</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3443,6 +4089,12 @@
       </c>
       <c r="F108" t="n">
         <v>1</v>
+      </c>
+      <c r="G108" t="n">
+        <v>40769696</v>
+      </c>
+      <c r="H108" t="n">
+        <v>79074334</v>
       </c>
     </row>
     <row r="109">
@@ -3462,7 +4114,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>39994</v>
+        <v>17555</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3471,6 +4123,12 @@
       </c>
       <c r="F109" t="n">
         <v>1</v>
+      </c>
+      <c r="G109" t="n">
+        <v>36111</v>
+      </c>
+      <c r="H109" t="n">
+        <v>64761</v>
       </c>
     </row>
     <row r="110">
@@ -3490,7 +4148,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>516672</v>
+        <v>114611</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3499,6 +4157,12 @@
       </c>
       <c r="F110" t="n">
         <v>1</v>
+      </c>
+      <c r="G110" t="n">
+        <v>254621</v>
+      </c>
+      <c r="H110" t="n">
+        <v>438765</v>
       </c>
     </row>
     <row r="111">
@@ -3518,7 +4182,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>19844</v>
+        <v>902903</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3527,6 +4191,12 @@
       </c>
       <c r="F111" t="n">
         <v>1</v>
+      </c>
+      <c r="G111" t="n">
+        <v>4227550</v>
+      </c>
+      <c r="H111" t="n">
+        <v>2245310</v>
       </c>
     </row>
     <row r="112">
@@ -3546,7 +4216,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>120836</v>
+        <v>76951</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3555,6 +4225,12 @@
       </c>
       <c r="F112" t="n">
         <v>1</v>
+      </c>
+      <c r="G112" t="n">
+        <v>167827</v>
+      </c>
+      <c r="H112" t="n">
+        <v>165348</v>
       </c>
     </row>
     <row r="113">
@@ -3574,7 +4250,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>76939</v>
+        <v>116874</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3583,6 +4259,12 @@
       </c>
       <c r="F113" t="n">
         <v>1</v>
+      </c>
+      <c r="G113" t="n">
+        <v>356812</v>
+      </c>
+      <c r="H113" t="n">
+        <v>568737</v>
       </c>
     </row>
     <row r="114">
@@ -3602,7 +4284,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>117084</v>
+        <v>1970602</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3611,6 +4293,12 @@
       </c>
       <c r="F114" t="n">
         <v>1</v>
+      </c>
+      <c r="G114" t="n">
+        <v>4212726</v>
+      </c>
+      <c r="H114" t="n">
+        <v>9041830</v>
       </c>
     </row>
     <row r="115">
@@ -3630,7 +4318,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>19820571</v>
+        <v>51744</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3639,6 +4327,12 @@
       </c>
       <c r="F115" t="n">
         <v>1</v>
+      </c>
+      <c r="G115" t="n">
+        <v>103709</v>
+      </c>
+      <c r="H115" t="n">
+        <v>146730</v>
       </c>
     </row>
     <row r="116">
@@ -3658,7 +4352,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>62081</v>
+        <v>459197</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3667,6 +4361,12 @@
       </c>
       <c r="F116" t="n">
         <v>1</v>
+      </c>
+      <c r="G116" t="n">
+        <v>2123358</v>
+      </c>
+      <c r="H116" t="n">
+        <v>1087666</v>
       </c>
     </row>
     <row r="117">
@@ -3686,7 +4386,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>8403</v>
+        <v>6363</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3695,6 +4395,12 @@
       </c>
       <c r="F117" t="n">
         <v>1</v>
+      </c>
+      <c r="G117" t="n">
+        <v>33520</v>
+      </c>
+      <c r="H117" t="n">
+        <v>12748</v>
       </c>
     </row>
     <row r="118">
@@ -3714,7 +4420,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>50330</v>
+        <v>1125001</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3723,6 +4429,12 @@
       </c>
       <c r="F118" t="n">
         <v>1</v>
+      </c>
+      <c r="G118" t="n">
+        <v>2351225</v>
+      </c>
+      <c r="H118" t="n">
+        <v>2885465</v>
       </c>
     </row>
     <row r="119">
@@ -3742,7 +4454,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>718050</v>
+        <v>31336</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3751,6 +4463,12 @@
       </c>
       <c r="F119" t="n">
         <v>1</v>
+      </c>
+      <c r="G119" t="n">
+        <v>182707</v>
+      </c>
+      <c r="H119" t="n">
+        <v>140586</v>
       </c>
     </row>
     <row r="120">
@@ -3770,7 +4488,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>3521307</v>
+        <v>74316</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3779,6 +4497,12 @@
       </c>
       <c r="F120" t="n">
         <v>1</v>
+      </c>
+      <c r="G120" t="n">
+        <v>361470</v>
+      </c>
+      <c r="H120" t="n">
+        <v>340130</v>
       </c>
     </row>
     <row r="121">
@@ -3798,7 +4522,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>931899</v>
+        <v>823234</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3807,6 +4531,12 @@
       </c>
       <c r="F121" t="n">
         <v>1</v>
+      </c>
+      <c r="G121" t="n">
+        <v>4019610</v>
+      </c>
+      <c r="H121" t="n">
+        <v>2658771</v>
       </c>
     </row>
   </sheetData>
@@ -3820,7 +4550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3854,6 +4584,16 @@
           <t>환율</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3872,7 +4612,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>339893</v>
+        <v>317247</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -3882,6 +4622,12 @@
       <c r="F2" t="n">
         <v>1300</v>
       </c>
+      <c r="G2" t="n">
+        <v>1190078</v>
+      </c>
+      <c r="H2" t="n">
+        <v>690060</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3900,7 +4646,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8760</v>
+        <v>1600778</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -3910,6 +4656,12 @@
       <c r="F3" t="n">
         <v>1300</v>
       </c>
+      <c r="G3" t="n">
+        <v>6951805</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4093559</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3928,7 +4680,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>9323</v>
+        <v>8698</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -3938,6 +4690,12 @@
       <c r="F4" t="n">
         <v>1300</v>
       </c>
+      <c r="G4" t="n">
+        <v>30828</v>
+      </c>
+      <c r="H4" t="n">
+        <v>48460</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3956,7 +4714,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>36511</v>
+        <v>18829</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -3965,6 +4723,12 @@
       </c>
       <c r="F5" t="n">
         <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>31002</v>
+      </c>
+      <c r="H5" t="n">
+        <v>85644</v>
       </c>
     </row>
     <row r="6">
@@ -3984,7 +4748,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>34527</v>
+        <v>5325</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -3993,6 +4757,12 @@
       </c>
       <c r="F6" t="n">
         <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>16399</v>
+      </c>
+      <c r="H6" t="n">
+        <v>11731</v>
       </c>
     </row>
     <row r="7">
@@ -4012,7 +4782,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>126025</v>
+        <v>7197</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -4021,6 +4791,12 @@
       </c>
       <c r="F7" t="n">
         <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>27940</v>
+      </c>
+      <c r="H7" t="n">
+        <v>28479</v>
       </c>
     </row>
     <row r="8">
@@ -4040,7 +4816,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1194741</v>
+        <v>5927</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -4049,6 +4825,12 @@
       </c>
       <c r="F8" t="n">
         <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>10345</v>
+      </c>
+      <c r="H8" t="n">
+        <v>33962</v>
       </c>
     </row>
     <row r="9">
@@ -4068,7 +4850,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7936</v>
+        <v>7445</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -4077,6 +4859,12 @@
       </c>
       <c r="F9" t="n">
         <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>12888</v>
+      </c>
+      <c r="H9" t="n">
+        <v>36830</v>
       </c>
     </row>
     <row r="10">
@@ -4096,7 +4884,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>59690</v>
+        <v>342766</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -4105,6 +4893,12 @@
       </c>
       <c r="F10" t="n">
         <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1529238</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1007437</v>
       </c>
     </row>
     <row r="11">
@@ -4124,7 +4918,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3634</v>
+        <v>25383</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -4133,6 +4927,12 @@
       </c>
       <c r="F11" t="n">
         <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>95815</v>
+      </c>
+      <c r="H11" t="n">
+        <v>97506</v>
       </c>
     </row>
     <row r="12">
@@ -4152,7 +4952,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1709753</v>
+        <v>615110</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -4161,6 +4961,12 @@
       </c>
       <c r="F12" t="n">
         <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2882794</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1937151</v>
       </c>
     </row>
     <row r="13">
@@ -4180,7 +4986,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>42521</v>
+        <v>7127</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -4189,6 +4995,12 @@
       </c>
       <c r="F13" t="n">
         <v>1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>26725</v>
+      </c>
+      <c r="H13" t="n">
+        <v>16463</v>
       </c>
     </row>
     <row r="14">
@@ -4208,7 +5020,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1485902</v>
+        <v>29930</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -4217,6 +5029,12 @@
       </c>
       <c r="F14" t="n">
         <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>113146</v>
+      </c>
+      <c r="H14" t="n">
+        <v>142811</v>
       </c>
     </row>
     <row r="15">
@@ -4236,7 +5054,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>146774</v>
+        <v>15561</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -4245,6 +5063,12 @@
       </c>
       <c r="F15" t="n">
         <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>26646</v>
+      </c>
+      <c r="H15" t="n">
+        <v>47852</v>
       </c>
     </row>
     <row r="16">
@@ -4264,7 +5088,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>15963</v>
+        <v>7691</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -4273,6 +5097,12 @@
       </c>
       <c r="F16" t="n">
         <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>29727</v>
+      </c>
+      <c r="H16" t="n">
+        <v>24331</v>
       </c>
     </row>
     <row r="17">
@@ -4292,7 +5122,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6449</v>
+        <v>239399</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -4301,6 +5131,12 @@
       </c>
       <c r="F17" t="n">
         <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>749842</v>
+      </c>
+      <c r="H17" t="n">
+        <v>592276</v>
       </c>
     </row>
     <row r="18">
@@ -4320,7 +5156,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>34521</v>
+        <v>29025</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -4329,6 +5165,12 @@
       </c>
       <c r="F18" t="n">
         <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>52260</v>
+      </c>
+      <c r="H18" t="n">
+        <v>112960</v>
       </c>
     </row>
     <row r="19">
@@ -4348,7 +5190,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>52177</v>
+        <v>237691</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -4357,6 +5199,12 @@
       </c>
       <c r="F19" t="n">
         <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1038626</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1395826</v>
       </c>
     </row>
     <row r="20">
@@ -4376,7 +5224,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>16260</v>
+        <v>1990950</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4385,6 +5233,12 @@
       </c>
       <c r="F20" t="n">
         <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>5682111</v>
+      </c>
+      <c r="H20" t="n">
+        <v>11281161</v>
       </c>
     </row>
     <row r="21">
@@ -4404,7 +5258,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>28183</v>
+        <v>18358</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4413,6 +5267,12 @@
       </c>
       <c r="F21" t="n">
         <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>33338</v>
+      </c>
+      <c r="H21" t="n">
+        <v>91603</v>
       </c>
     </row>
     <row r="22">
@@ -4432,7 +5292,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>49366</v>
+        <v>385822</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4441,6 +5301,12 @@
       </c>
       <c r="F22" t="n">
         <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>757800</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2037476</v>
       </c>
     </row>
     <row r="23">
@@ -4460,7 +5326,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>177809</v>
+        <v>366059</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4469,6 +5335,12 @@
       </c>
       <c r="F23" t="n">
         <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1450207</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1070917</v>
       </c>
     </row>
     <row r="24">
@@ -4488,7 +5360,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1751292</v>
+        <v>1091121</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4497,6 +5369,12 @@
       </c>
       <c r="F24" t="n">
         <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2244139</v>
+      </c>
+      <c r="H24" t="n">
+        <v>6328324</v>
       </c>
     </row>
     <row r="25">
@@ -4516,7 +5394,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9325</v>
+        <v>1108129</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4525,6 +5403,12 @@
       </c>
       <c r="F25" t="n">
         <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4482537</v>
+      </c>
+      <c r="H25" t="n">
+        <v>4060988</v>
       </c>
     </row>
     <row r="26">
@@ -4544,7 +5428,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>369311</v>
+        <v>974117</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4553,6 +5437,12 @@
       </c>
       <c r="F26" t="n">
         <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4325867</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1955019</v>
       </c>
     </row>
     <row r="27">
@@ -4572,7 +5462,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1740710</v>
+        <v>351733</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4581,6 +5471,12 @@
       </c>
       <c r="F27" t="n">
         <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>675379</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2006848</v>
       </c>
     </row>
     <row r="28">
@@ -4600,7 +5496,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>38932</v>
+        <v>9262</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4609,6 +5505,12 @@
       </c>
       <c r="F28" t="n">
         <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>23288</v>
+      </c>
+      <c r="H28" t="n">
+        <v>32313</v>
       </c>
     </row>
     <row r="29">
@@ -4628,7 +5530,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9046</v>
+        <v>1085242</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4637,6 +5539,12 @@
       </c>
       <c r="F29" t="n">
         <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4932316</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2502136</v>
       </c>
     </row>
     <row r="30">
@@ -4656,7 +5564,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>42385</v>
+        <v>1633485</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -4665,6 +5573,12 @@
       </c>
       <c r="F30" t="n">
         <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>7334172</v>
+      </c>
+      <c r="H30" t="n">
+        <v>5100639</v>
       </c>
     </row>
     <row r="31">
@@ -4684,7 +5598,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>22756</v>
+        <v>8760</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4693,6 +5607,12 @@
       </c>
       <c r="F31" t="n">
         <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>21897</v>
+      </c>
+      <c r="H31" t="n">
+        <v>50303</v>
       </c>
     </row>
     <row r="32">
@@ -4712,7 +5632,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1428652</v>
+        <v>58697</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -4721,6 +5641,12 @@
       </c>
       <c r="F32" t="n">
         <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>177666</v>
+      </c>
+      <c r="H32" t="n">
+        <v>191493</v>
       </c>
     </row>
     <row r="33">
@@ -4740,7 +5666,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6674</v>
+        <v>335543</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -4749,6 +5675,12 @@
       </c>
       <c r="F33" t="n">
         <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1005661</v>
+      </c>
+      <c r="H33" t="n">
+        <v>710024</v>
       </c>
     </row>
     <row r="34">
@@ -4768,7 +5700,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>304699</v>
+        <v>1870136</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -4777,6 +5709,12 @@
       </c>
       <c r="F34" t="n">
         <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>8962528</v>
+      </c>
+      <c r="H34" t="n">
+        <v>7848797</v>
       </c>
     </row>
     <row r="35">
@@ -4796,7 +5734,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1676409</v>
+        <v>2871</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -4805,6 +5743,12 @@
       </c>
       <c r="F35" t="n">
         <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>11666</v>
+      </c>
+      <c r="H35" t="n">
+        <v>10920</v>
       </c>
     </row>
     <row r="36">
@@ -4824,7 +5768,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9124</v>
+        <v>44002</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -4833,6 +5777,12 @@
       </c>
       <c r="F36" t="n">
         <v>1</v>
+      </c>
+      <c r="G36" t="n">
+        <v>110081</v>
+      </c>
+      <c r="H36" t="n">
+        <v>96625</v>
       </c>
     </row>
     <row r="37">
@@ -4852,7 +5802,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4364</v>
+        <v>22684</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -4861,6 +5811,12 @@
       </c>
       <c r="F37" t="n">
         <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>66965</v>
+      </c>
+      <c r="H37" t="n">
+        <v>70934</v>
       </c>
     </row>
     <row r="38">
@@ -4880,7 +5836,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>112660</v>
+        <v>321710</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -4889,6 +5845,12 @@
       </c>
       <c r="F38" t="n">
         <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1581859</v>
+      </c>
+      <c r="H38" t="n">
+        <v>978215</v>
       </c>
     </row>
     <row r="39">
@@ -4908,7 +5870,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6308</v>
+        <v>28538</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -4917,6 +5879,12 @@
       </c>
       <c r="F39" t="n">
         <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>98473</v>
+      </c>
+      <c r="H39" t="n">
+        <v>102093</v>
       </c>
     </row>
     <row r="40">
@@ -4936,7 +5904,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8200</v>
+        <v>43944</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -4945,6 +5913,12 @@
       </c>
       <c r="F40" t="n">
         <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>77478</v>
+      </c>
+      <c r="H40" t="n">
+        <v>175883</v>
       </c>
     </row>
     <row r="41">
@@ -4964,7 +5938,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>5824</v>
+        <v>1325580</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -4973,6 +5947,12 @@
       </c>
       <c r="F41" t="n">
         <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>4090012</v>
+      </c>
+      <c r="H41" t="n">
+        <v>4415953</v>
       </c>
     </row>
     <row r="42">
@@ -4992,7 +5972,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>46173</v>
+        <v>1141135</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -5001,6 +5981,12 @@
       </c>
       <c r="F42" t="n">
         <v>1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>3899540</v>
+      </c>
+      <c r="H42" t="n">
+        <v>3396407</v>
       </c>
     </row>
     <row r="43">
@@ -5020,7 +6006,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1262234</v>
+        <v>30388</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -5029,6 +6015,12 @@
       </c>
       <c r="F43" t="n">
         <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>55271</v>
+      </c>
+      <c r="H43" t="n">
+        <v>89842</v>
       </c>
     </row>
     <row r="44">
@@ -5048,7 +6040,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1261628</v>
+        <v>342808</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -5057,6 +6049,12 @@
       </c>
       <c r="F44" t="n">
         <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>756746</v>
+      </c>
+      <c r="H44" t="n">
+        <v>713152</v>
       </c>
     </row>
     <row r="45">
@@ -5076,7 +6074,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>46465</v>
+        <v>1074257</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -5085,6 +6083,12 @@
       </c>
       <c r="F45" t="n">
         <v>1</v>
+      </c>
+      <c r="G45" t="n">
+        <v>4415670</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3050911</v>
       </c>
     </row>
     <row r="46">
@@ -5104,7 +6108,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>376835</v>
+        <v>201461</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -5113,6 +6117,12 @@
       </c>
       <c r="F46" t="n">
         <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>345950</v>
+      </c>
+      <c r="H46" t="n">
+        <v>626557</v>
       </c>
     </row>
     <row r="47">
@@ -5132,7 +6142,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>52800</v>
+        <v>137762</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -5141,6 +6151,12 @@
       </c>
       <c r="F47" t="n">
         <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>449364</v>
+      </c>
+      <c r="H47" t="n">
+        <v>622479</v>
       </c>
     </row>
     <row r="48">
@@ -5160,7 +6176,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>33749</v>
+        <v>19167</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -5169,6 +6185,12 @@
       </c>
       <c r="F48" t="n">
         <v>1</v>
+      </c>
+      <c r="G48" t="n">
+        <v>88911</v>
+      </c>
+      <c r="H48" t="n">
+        <v>67817</v>
       </c>
     </row>
     <row r="49">
@@ -5188,7 +6210,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1163177</v>
+        <v>1147755</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -5197,6 +6219,12 @@
       </c>
       <c r="F49" t="n">
         <v>1</v>
+      </c>
+      <c r="G49" t="n">
+        <v>2975045</v>
+      </c>
+      <c r="H49" t="n">
+        <v>6034157</v>
       </c>
     </row>
     <row r="50">
@@ -5216,7 +6244,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>7534</v>
+        <v>3454</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -5225,6 +6253,12 @@
       </c>
       <c r="F50" t="n">
         <v>1</v>
+      </c>
+      <c r="G50" t="n">
+        <v>10322</v>
+      </c>
+      <c r="H50" t="n">
+        <v>17461</v>
       </c>
     </row>
     <row r="51">
@@ -5244,7 +6278,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>609681</v>
+        <v>1952422</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -5253,6 +6287,12 @@
       </c>
       <c r="F51" t="n">
         <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>6275836</v>
+      </c>
+      <c r="H51" t="n">
+        <v>4476028</v>
       </c>
     </row>
     <row r="52">
@@ -5272,7 +6312,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>335181</v>
+        <v>1958362</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -5281,6 +6321,12 @@
       </c>
       <c r="F52" t="n">
         <v>1</v>
+      </c>
+      <c r="G52" t="n">
+        <v>4640590</v>
+      </c>
+      <c r="H52" t="n">
+        <v>4770929</v>
       </c>
     </row>
     <row r="53">
@@ -5300,7 +6346,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>57278</v>
+        <v>21843</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -5309,6 +6355,12 @@
       </c>
       <c r="F53" t="n">
         <v>1</v>
+      </c>
+      <c r="G53" t="n">
+        <v>107066</v>
+      </c>
+      <c r="H53" t="n">
+        <v>53200</v>
       </c>
     </row>
     <row r="54">
@@ -5328,7 +6380,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>142894</v>
+        <v>627505</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -5337,6 +6389,12 @@
       </c>
       <c r="F54" t="n">
         <v>1</v>
+      </c>
+      <c r="G54" t="n">
+        <v>2647454</v>
+      </c>
+      <c r="H54" t="n">
+        <v>1258439</v>
       </c>
     </row>
     <row r="55">
@@ -5356,7 +6414,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>58540</v>
+        <v>25466</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -5365,6 +6423,12 @@
       </c>
       <c r="F55" t="n">
         <v>1</v>
+      </c>
+      <c r="G55" t="n">
+        <v>120192</v>
+      </c>
+      <c r="H55" t="n">
+        <v>116686</v>
       </c>
     </row>
     <row r="56">
@@ -5384,7 +6448,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>48601</v>
+        <v>388730</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -5393,6 +6457,12 @@
       </c>
       <c r="F56" t="n">
         <v>1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1435447</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1598853</v>
       </c>
     </row>
     <row r="57">
@@ -5412,7 +6482,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5487</v>
+        <v>1547873</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -5421,6 +6491,12 @@
       </c>
       <c r="F57" t="n">
         <v>1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>2929294</v>
+      </c>
+      <c r="H57" t="n">
+        <v>3531329</v>
       </c>
     </row>
     <row r="58">
@@ -5440,7 +6516,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>744193</v>
+        <v>32464</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -5449,6 +6525,12 @@
       </c>
       <c r="F58" t="n">
         <v>1</v>
+      </c>
+      <c r="G58" t="n">
+        <v>74100</v>
+      </c>
+      <c r="H58" t="n">
+        <v>142978</v>
       </c>
     </row>
     <row r="59">
@@ -5468,7 +6550,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>22266</v>
+        <v>6531</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -5477,6 +6559,12 @@
       </c>
       <c r="F59" t="n">
         <v>1</v>
+      </c>
+      <c r="G59" t="n">
+        <v>32572</v>
+      </c>
+      <c r="H59" t="n">
+        <v>20340</v>
       </c>
     </row>
     <row r="60">
@@ -5496,7 +6584,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1991109</v>
+        <v>293373</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -5505,6 +6593,12 @@
       </c>
       <c r="F60" t="n">
         <v>1</v>
+      </c>
+      <c r="G60" t="n">
+        <v>1347522</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1144510</v>
       </c>
     </row>
     <row r="61">
@@ -5524,7 +6618,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1008674</v>
+        <v>39615</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -5533,6 +6627,12 @@
       </c>
       <c r="F61" t="n">
         <v>1</v>
+      </c>
+      <c r="G61" t="n">
+        <v>63483</v>
+      </c>
+      <c r="H61" t="n">
+        <v>144486</v>
       </c>
     </row>
     <row r="62">
@@ -5552,7 +6652,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>31048</v>
+        <v>116593</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -5561,6 +6661,12 @@
       </c>
       <c r="F62" t="n">
         <v>1</v>
+      </c>
+      <c r="G62" t="n">
+        <v>254102</v>
+      </c>
+      <c r="H62" t="n">
+        <v>645852</v>
       </c>
     </row>
     <row r="63">
@@ -5580,7 +6686,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>7916</v>
+        <v>621638</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -5589,6 +6695,12 @@
       </c>
       <c r="F63" t="n">
         <v>1</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1428177</v>
+      </c>
+      <c r="H63" t="n">
+        <v>2298376</v>
       </c>
     </row>
     <row r="64">
@@ -5608,7 +6720,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5035</v>
+        <v>168036</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -5617,6 +6729,12 @@
       </c>
       <c r="F64" t="n">
         <v>1</v>
+      </c>
+      <c r="G64" t="n">
+        <v>272107</v>
+      </c>
+      <c r="H64" t="n">
+        <v>563291</v>
       </c>
     </row>
     <row r="65">
@@ -5636,7 +6754,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1160687</v>
+        <v>1043480</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -5645,6 +6763,12 @@
       </c>
       <c r="F65" t="n">
         <v>1</v>
+      </c>
+      <c r="G65" t="n">
+        <v>3012791</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2115148</v>
       </c>
     </row>
     <row r="66">
@@ -5664,7 +6788,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>5383</v>
+        <v>321739</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -5673,6 +6797,12 @@
       </c>
       <c r="F66" t="n">
         <v>1</v>
+      </c>
+      <c r="G66" t="n">
+        <v>1051144</v>
+      </c>
+      <c r="H66" t="n">
+        <v>907585</v>
       </c>
     </row>
     <row r="67">
@@ -5692,7 +6822,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>253679</v>
+        <v>29027</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -5701,6 +6831,12 @@
       </c>
       <c r="F67" t="n">
         <v>1</v>
+      </c>
+      <c r="G67" t="n">
+        <v>126849</v>
+      </c>
+      <c r="H67" t="n">
+        <v>84853</v>
       </c>
     </row>
     <row r="68">
@@ -5720,7 +6856,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>3346</v>
+        <v>26926</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -5729,6 +6865,12 @@
       </c>
       <c r="F68" t="n">
         <v>1</v>
+      </c>
+      <c r="G68" t="n">
+        <v>124201</v>
+      </c>
+      <c r="H68" t="n">
+        <v>65593</v>
       </c>
     </row>
     <row r="69">
@@ -5748,7 +6890,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>58726</v>
+        <v>1415147</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -5757,6 +6899,12 @@
       </c>
       <c r="F69" t="n">
         <v>1</v>
+      </c>
+      <c r="G69" t="n">
+        <v>6562982</v>
+      </c>
+      <c r="H69" t="n">
+        <v>5575980</v>
       </c>
     </row>
     <row r="70">
@@ -5776,7 +6924,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>3130</v>
+        <v>9616</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -5785,6 +6933,12 @@
       </c>
       <c r="F70" t="n">
         <v>1</v>
+      </c>
+      <c r="G70" t="n">
+        <v>19350</v>
+      </c>
+      <c r="H70" t="n">
+        <v>34365</v>
       </c>
     </row>
     <row r="71">
@@ -5804,7 +6958,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>111876</v>
+        <v>16063</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -5813,6 +6967,12 @@
       </c>
       <c r="F71" t="n">
         <v>1</v>
+      </c>
+      <c r="G71" t="n">
+        <v>57610</v>
+      </c>
+      <c r="H71" t="n">
+        <v>58816</v>
       </c>
     </row>
     <row r="72">
@@ -5832,7 +6992,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>27170</v>
+        <v>3881</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -5841,6 +7001,12 @@
       </c>
       <c r="F72" t="n">
         <v>1</v>
+      </c>
+      <c r="G72" t="n">
+        <v>11929</v>
+      </c>
+      <c r="H72" t="n">
+        <v>18815</v>
       </c>
     </row>
     <row r="73">
@@ -5860,7 +7026,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>51890</v>
+        <v>319817</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -5869,6 +7035,12 @@
       </c>
       <c r="F73" t="n">
         <v>1</v>
+      </c>
+      <c r="G73" t="n">
+        <v>1596321</v>
+      </c>
+      <c r="H73" t="n">
+        <v>1831395</v>
       </c>
     </row>
     <row r="74">
@@ -5888,7 +7060,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>221784</v>
+        <v>157205</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -5897,6 +7069,12 @@
       </c>
       <c r="F74" t="n">
         <v>1</v>
+      </c>
+      <c r="G74" t="n">
+        <v>594807</v>
+      </c>
+      <c r="H74" t="n">
+        <v>644413</v>
       </c>
     </row>
     <row r="75">
@@ -5916,7 +7094,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1550626</v>
+        <v>547841</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -5925,6 +7103,12 @@
       </c>
       <c r="F75" t="n">
         <v>1</v>
+      </c>
+      <c r="G75" t="n">
+        <v>2095766</v>
+      </c>
+      <c r="H75" t="n">
+        <v>1925373</v>
       </c>
     </row>
     <row r="76">
@@ -5944,7 +7128,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4593</v>
+        <v>395495</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -5953,6 +7137,12 @@
       </c>
       <c r="F76" t="n">
         <v>1</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1205675</v>
+      </c>
+      <c r="H76" t="n">
+        <v>963358</v>
       </c>
     </row>
     <row r="77">
@@ -5972,7 +7162,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>34139</v>
+        <v>4599</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -5981,6 +7171,12 @@
       </c>
       <c r="F77" t="n">
         <v>1</v>
+      </c>
+      <c r="G77" t="n">
+        <v>12555</v>
+      </c>
+      <c r="H77" t="n">
+        <v>26773</v>
       </c>
     </row>
     <row r="78">
@@ -6000,7 +7196,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>4517</v>
+        <v>6708</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -6009,6 +7205,12 @@
       </c>
       <c r="F78" t="n">
         <v>1</v>
+      </c>
+      <c r="G78" t="n">
+        <v>27879</v>
+      </c>
+      <c r="H78" t="n">
+        <v>23617</v>
       </c>
     </row>
     <row r="79">
@@ -6028,7 +7230,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>7258</v>
+        <v>346602</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -6037,6 +7239,12 @@
       </c>
       <c r="F79" t="n">
         <v>1</v>
+      </c>
+      <c r="G79" t="n">
+        <v>1044512</v>
+      </c>
+      <c r="H79" t="n">
+        <v>761496</v>
       </c>
     </row>
     <row r="80">
@@ -6056,7 +7264,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>125123</v>
+        <v>793574</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -6065,6 +7273,12 @@
       </c>
       <c r="F80" t="n">
         <v>1</v>
+      </c>
+      <c r="G80" t="n">
+        <v>2694462</v>
+      </c>
+      <c r="H80" t="n">
+        <v>3003986</v>
       </c>
     </row>
     <row r="81">
@@ -6084,7 +7298,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>17998</v>
+        <v>209275</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -6093,6 +7307,12 @@
       </c>
       <c r="F81" t="n">
         <v>1</v>
+      </c>
+      <c r="G81" t="n">
+        <v>970925</v>
+      </c>
+      <c r="H81" t="n">
+        <v>443898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>